<commit_message>
F-LA-03: puntos de control / vértices con número fijo (repeat_count)
El repeat «Puntos de control / vértices del predio» (r_puntos) era abierto:
Kobo pedía agregar puntos sin fin y no dejaba seguir con el formulario ni
volver al inicio. Ahora se pregunta antes cuántos puntos se registrarán
(n_puntos, 0 a 50) y el repeat usa repeat_count: se llenan solo esos puntos
y el formulario continúa. Mismo cambio en la Ficha técnica predial completa.

- la_campos.Repeat.max_filas; r_puntos de F-LA-03 con max_filas=50
- la_plantillas: campo n_… + repeat_count en el XLSForm; columna repeat_count
- la_xlsform_ficha: n_puntos + repeat_count; XLSForm FP regenerado
- LEEME de ambos paquetes y pruebas de regresión

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011TLfW3Dq6Rn7SD1KppDuzJ
</commit_message>
<xml_diff>
--- a/kobo_ficha_predial/FP_Ficha_Predial_Completa_KOBO.xlsx
+++ b/kobo_ficha_predial/FP_Ficha_Predial_Completa_KOBO.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M162"/>
+  <dimension ref="A1:N163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -442,6 +442,7 @@
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -510,6 +511,11 @@
           <t>parameters</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>repeat_count</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3511,117 +3517,142 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>begin_repeat</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>r_puntos</t>
+          <t>n_puntos</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Puntos de control / vértices del predio</t>
+          <t>N.° de puntos de control / vértices del predio</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Indique cuántos registrará (0 a 50). Para corregir, vuelva aquí y cambie el número.</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 50</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Entre 0 y 50</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>geopoint</t>
+          <t>begin_repeat</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>pt_gps</t>
+          <t>r_puntos</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Punto</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>Precisión ≤ 10 m.</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Puntos de control / vértices del predio</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>${n_puntos} &gt; 0</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>${n_puntos}</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>select_one pt_tipo</t>
+          <t>geopoint</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>pt_tipo</t>
+          <t>pt_gps</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Tipo de punto</t>
+          <t>Punto</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Precisión ≤ 10 m.</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>end_repeat</t>
+          <t>select_one pt_tipo</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>r_puntos</t>
+          <t>pt_tipo</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Tipo de punto</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>end_repeat</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>g_fotos</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>8. Panel fotográfico</t>
+          <t>r_puntos</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>foto_1</t>
+          <t>g_fotos</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Foto 1 – Vista general del predio</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>Tome la foto con la cámara del celular (o elija una imagen).</t>
-        </is>
-      </c>
-      <c r="M153" t="inlineStr">
-        <is>
-          <t>max-pixels=1280</t>
+          <t>8. Panel fotográfico</t>
         </is>
       </c>
     </row>
@@ -3633,12 +3664,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>foto_2</t>
+          <t>foto_1</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Foto 2 – Cobertura vegetal / uso actual</t>
+          <t>Foto 1 – Vista general del predio</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -3660,12 +3691,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>foto_3</t>
+          <t>foto_2</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Foto 3 – Linderos, hitos o accesos</t>
+          <t>Foto 2 – Cobertura vegetal / uso actual</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -3687,12 +3718,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>foto_4</t>
+          <t>foto_3</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Foto 4 – Interferencias o detalle relevante</t>
+          <t>Foto 3 – Linderos, hitos o accesos</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -3709,110 +3740,137 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>g_fotos</t>
+          <t>foto_4</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Foto 4 – Interferencias o detalle relevante</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Tome la foto con la cámara del celular (o elija una imagen).</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>max-pixels=1280</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>end_group</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>g_firmas</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>9. Conformidad</t>
+          <t>g_fotos</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>firma_prediante</t>
+          <t>g_firmas</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Firma del prediante / titular (conformidad)</t>
-        </is>
-      </c>
-      <c r="F159" t="inlineStr">
-        <is>
-          <t>${consentimiento}='si'</t>
-        </is>
-      </c>
-      <c r="K159" t="inlineStr">
-        <is>
-          <t>signature</t>
-        </is>
-      </c>
-      <c r="M159" t="inlineStr">
-        <is>
-          <t>max-pixels=800</t>
+          <t>9. Conformidad</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>lugar</t>
+          <t>firma_prediante</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Lugar</t>
+          <t>Firma del prediante / titular (conformidad)</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>${consentimiento}='si'</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>signature</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>max-pixels=800</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>g_firmas</t>
+          <t>lugar</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Lugar</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>g_firmas</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr">
+      <c r="B163" t="inlineStr">
         <is>
           <t>nota_fin</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr">
+      <c r="C163" t="inlineStr">
         <is>
           <t>Fin de la ficha predial. Pulse «Enviar»: el formulario queda en blanco y vuelve al inicio para registrar el siguiente predio.</t>
         </is>
       </c>
-      <c r="D162" t="inlineStr">
+      <c r="D163" t="inlineStr">
         <is>
           <t>Use el enlace «En línea-Fuera de línea (envíos múltiples)» de KoboToolbox o KoboCollect.</t>
         </is>
@@ -7328,7 +7386,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>202610260022</t>
+          <t>202610271747</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>

<commit_message>
F-LA-04 y Ficha predial: firmantes y afectaciones con número fijo
Mismo arreglo que r_puntos para los otros dos repeats abiertos, donde Kobo
pedía filas sin fin y no dejaba seguir con el formulario:
- F-LA-04 r_firmantes: n_firmantes (0 a 200) + repeat_count
- Ficha predial completa r_afectaciones: n_afectaciones (1 a 20, solo si hay
  afectaciones) + repeat_count; XLSForm FP regenerado
- LEEME actualizados; pruebas: ningún formulario Kobo queda con repeat abierto

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011TLfW3Dq6Rn7SD1KppDuzJ
</commit_message>
<xml_diff>
--- a/kobo_ficha_predial/FP_Ficha_Predial_Completa_KOBO.xlsx
+++ b/kobo_ficha_predial/FP_Ficha_Predial_Completa_KOBO.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N163"/>
+  <dimension ref="A1:N164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3086,341 +3086,366 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>begin_repeat</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>r_afectaciones</t>
+          <t>n_afectaciones</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Afectaciones (OC-01, OC-02…)</t>
+          <t>N.° de obras o bienes afectados</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Indique cuántos registrará (1 a 20). Para corregir, vuelva aquí y cambie el número.</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
           <t>${tiene_afectaciones}='si'</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 20</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Entre 1 y 20</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>begin_repeat</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>af_codigo</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>concat('OC-', if(position(..) &lt; 10, '0', ''), position(..))</t>
+          <t>r_afectaciones</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Afectaciones (OC-01, OC-02…)</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>${tiene_afectaciones}='si' and ${n_afectaciones} &gt; 0</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>${n_afectaciones}</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>calculate</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>af_nota</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>**${af_codigo}**</t>
+          <t>af_codigo</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>concat('OC-', if(position(..) &lt; 10, '0', ''), position(..))</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>af_descripcion</t>
+          <t>af_nota</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Descripción / uso</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>**${af_codigo}**</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>af_metrado</t>
+          <t>af_descripcion</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Metrado</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>. &gt;= 0</t>
-        </is>
-      </c>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>Valor no negativo</t>
+          <t>Descripción / uso</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>select_one und_medida</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>af_und</t>
+          <t>af_metrado</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Unidad de medida</t>
+          <t>Metrado</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>. &gt;= 0</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Valor no negativo</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>select_one material</t>
+          <t>select_one und_medida</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>af_material</t>
+          <t>af_und</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Material predominante</t>
+          <t>Unidad de medida</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>select_one conservacion</t>
+          <t>select_one material</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>af_conservacion</t>
+          <t>af_material</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Estado de conservación</t>
+          <t>Material predominante</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>select_one construccion</t>
+          <t>select_one conservacion</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>af_construccion</t>
+          <t>af_conservacion</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Estado de construcción</t>
+          <t>Estado de conservación</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one construccion</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>af_ubicacion</t>
+          <t>af_construccion</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Ubicación en el predio</t>
+          <t>Estado de construcción</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>end_repeat</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>r_afectaciones</t>
+          <t>af_ubicacion</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Ubicación en el predio</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>end_repeat</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>g_liberacion</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>6. Disponibilidad y condición de liberación</t>
+          <t>r_afectaciones</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>select_one aceptacion</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>aceptacion</t>
+          <t>g_liberacion</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Aceptación del titular / prediante</t>
-        </is>
-      </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>6. Disponibilidad y condición de liberación</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>select_one modalidad</t>
+          <t>select_one aceptacion</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>modalidad</t>
+          <t>aceptacion</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Modalidad de disponibilidad</t>
+          <t>Aceptación del titular / prediante</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>select_one conclusion_campo</t>
+          <t>select_one modalidad</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>conclusion_campo</t>
+          <t>modalidad</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Conclusión de campo</t>
-        </is>
-      </c>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Modalidad de disponibilidad</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>select_one estado_la</t>
+          <t>select_one conclusion_campo</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>estado_la_propuesto</t>
+          <t>conclusion_campo</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Estado LA propuesto</t>
+          <t>Conclusión de campo</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>select_one tipo_acta</t>
+          <t>select_one estado_la</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>tipo_acta_prevista</t>
+          <t>estado_la_propuesto</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Acta prevista</t>
+          <t>Estado LA propuesto</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one tipo_acta</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>cod_titular_prev</t>
+          <t>tipo_acta_prevista</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Código de titular ya registrado (T0000), si existe</t>
-        </is>
-      </c>
-      <c r="G142" t="inlineStr">
-        <is>
-          <t>regex(., '^T[0-9]{4}$')</t>
-        </is>
-      </c>
-      <c r="H142" t="inlineStr">
-        <is>
-          <t>Formato T0000 (T y 4 dígitos)</t>
+          <t>Acta prevista</t>
         </is>
       </c>
     </row>
@@ -3432,254 +3457,254 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>alertas</t>
+          <t>cod_titular_prev</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Observaciones / alertas sociales</t>
-        </is>
-      </c>
-      <c r="K143" t="inlineStr">
-        <is>
-          <t>multiline</t>
+          <t>Código de titular ya registrado (T0000), si existe</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>regex(., '^T[0-9]{4}$')</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Formato T0000 (T y 4 dígitos)</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>g_liberacion</t>
+          <t>alertas</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Observaciones / alertas sociales</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>multiline</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>end_group</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>g_croquis</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>7. Croquis del predio y puntos de control</t>
+          <t>g_liberacion</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>croquis</t>
+          <t>g_croquis</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Croquis del predio (dibuje: norte, linderos, accesos, vértices)</t>
-        </is>
-      </c>
-      <c r="K146" t="inlineStr">
-        <is>
-          <t>draw</t>
-        </is>
-      </c>
-      <c r="M146" t="inlineStr">
-        <is>
-          <t>max-pixels=1280</t>
+          <t>7. Croquis del predio y puntos de control</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>g_croquis</t>
+          <t>croquis</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Croquis del predio (dibuje: norte, linderos, accesos, vértices)</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>draw</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>max-pixels=1280</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>end_group</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>n_puntos</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>N.° de puntos de control / vértices del predio</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>Indique cuántos registrará (0 a 50). Para corregir, vuelva aquí y cambie el número.</t>
-        </is>
-      </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr">
-        <is>
-          <t>. &gt;= 0 and . &lt;= 50</t>
-        </is>
-      </c>
-      <c r="H148" t="inlineStr">
-        <is>
-          <t>Entre 0 y 50</t>
-        </is>
-      </c>
-      <c r="L148" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>g_croquis</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>begin_repeat</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>r_puntos</t>
+          <t>n_puntos</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Puntos de control / vértices del predio</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>${n_puntos} &gt; 0</t>
-        </is>
-      </c>
-      <c r="N149" t="inlineStr">
-        <is>
-          <t>${n_puntos}</t>
+          <t>N.° de puntos de control / vértices del predio</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Indique cuántos registrará (0 a 50). Para corregir, vuelva aquí y cambie el número.</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 50</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Entre 0 y 50</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>geopoint</t>
+          <t>begin_repeat</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>pt_gps</t>
+          <t>r_puntos</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Punto</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>Precisión ≤ 10 m.</t>
-        </is>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>yes</t>
+          <t>Puntos de control / vértices del predio</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>${n_puntos} &gt; 0</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>${n_puntos}</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>select_one pt_tipo</t>
+          <t>geopoint</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>pt_tipo</t>
+          <t>pt_gps</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Tipo de punto</t>
+          <t>Punto</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Precisión ≤ 10 m.</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>end_repeat</t>
+          <t>select_one pt_tipo</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>r_puntos</t>
+          <t>pt_tipo</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Tipo de punto</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>end_repeat</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>g_fotos</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>8. Panel fotográfico</t>
+          <t>r_puntos</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>foto_1</t>
+          <t>g_fotos</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Foto 1 – Vista general del predio</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>Tome la foto con la cámara del celular (o elija una imagen).</t>
-        </is>
-      </c>
-      <c r="M154" t="inlineStr">
-        <is>
-          <t>max-pixels=1280</t>
+          <t>8. Panel fotográfico</t>
         </is>
       </c>
     </row>
@@ -3691,12 +3716,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>foto_2</t>
+          <t>foto_1</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Foto 2 – Cobertura vegetal / uso actual</t>
+          <t>Foto 1 – Vista general del predio</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -3718,12 +3743,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>foto_3</t>
+          <t>foto_2</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Foto 3 – Linderos, hitos o accesos</t>
+          <t>Foto 2 – Cobertura vegetal / uso actual</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -3745,12 +3770,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>foto_4</t>
+          <t>foto_3</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Foto 4 – Interferencias o detalle relevante</t>
+          <t>Foto 3 – Linderos, hitos o accesos</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -3767,110 +3792,137 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>g_fotos</t>
+          <t>foto_4</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Foto 4 – Interferencias o detalle relevante</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Tome la foto con la cámara del celular (o elija una imagen).</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>max-pixels=1280</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>end_group</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>g_firmas</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>9. Conformidad</t>
+          <t>g_fotos</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>firma_prediante</t>
+          <t>g_firmas</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Firma del prediante / titular (conformidad)</t>
-        </is>
-      </c>
-      <c r="F160" t="inlineStr">
-        <is>
-          <t>${consentimiento}='si'</t>
-        </is>
-      </c>
-      <c r="K160" t="inlineStr">
-        <is>
-          <t>signature</t>
-        </is>
-      </c>
-      <c r="M160" t="inlineStr">
-        <is>
-          <t>max-pixels=800</t>
+          <t>9. Conformidad</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>lugar</t>
+          <t>firma_prediante</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Lugar</t>
+          <t>Firma del prediante / titular (conformidad)</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>${consentimiento}='si'</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>signature</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>max-pixels=800</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>end_group</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>g_firmas</t>
+          <t>lugar</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Lugar</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>g_firmas</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
           <t>note</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr">
+      <c r="B164" t="inlineStr">
         <is>
           <t>nota_fin</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
+      <c r="C164" t="inlineStr">
         <is>
           <t>Fin de la ficha predial. Pulse «Enviar»: el formulario queda en blanco y vuelve al inicio para registrar el siguiente predio.</t>
         </is>
       </c>
-      <c r="D163" t="inlineStr">
+      <c r="D164" t="inlineStr">
         <is>
           <t>Use el enlace «En línea-Fuera de línea (envíos múltiples)» de KoboToolbox o KoboCollect.</t>
         </is>
@@ -7386,7 +7438,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>202610271747</t>
+          <t>202610271828</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>